<commit_message>
Thiet ke trang luyen de v18
</commit_message>
<xml_diff>
--- a/ETS2023_Test2_Final_Architecture.xlsx
+++ b/ETS2023_Test2_Final_Architecture.xlsx
@@ -2839,9 +2839,6 @@
     <t>Giải thích: Chỗ trống đứng trước danh từ "salaries" (mức lương) nên cần một tính từ. "competitive" (cạnh tranh) ghép với salaries mang nghĩa "mức lương cạnh tranh / hấp dẫn".&lt;br&gt;Dịch nghĩa: Chúng tôi đưa ra mức lương cạnh tranh và các phúc lợi tuyệt vời.</t>
   </si>
   <si>
-    <t>https://github.com/bangvang1105-tech/Audio-Test-1-ETS-2023/raw/refs/heads/main/Test%202%20ETS%202023.mp3</t>
-  </si>
-  <si>
     <t>147</t>
   </si>
   <si>
@@ -4079,6 +4076,9 @@
   </si>
   <si>
     <t>https://raw.githubusercontent.com/bangvang1105-tech/Image-Test-2-ETS-2023/refs/heads/main/p7_186(1).png | https://raw.githubusercontent.com/bangvang1105-tech/Image-Test-2-ETS-2023/refs/heads/main/p7_186(2).png | https://raw.githubusercontent.com/bangvang1105-tech/Image-Test-2-ETS-2023/refs/heads/main/p7_186(3).png</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/uc?export=view&amp;id=14yGl8HQLGWVQRJ9wKb3tllrgH0prTzdC</t>
   </si>
 </sst>
 </file>
@@ -4551,7 +4551,7 @@
         <v>96</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>939</v>
+        <v>1352</v>
       </c>
       <c r="D2" s="2">
         <v>120</v>
@@ -4635,7 +4635,7 @@
         <v>18</v>
       </c>
       <c r="E2" s="8" t="s">
-        <v>1323</v>
+        <v>1322</v>
       </c>
       <c r="H2" s="5" t="s">
         <v>98</v>
@@ -4667,7 +4667,7 @@
         <v>20</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>1324</v>
+        <v>1323</v>
       </c>
       <c r="H3" s="5" t="s">
         <v>103</v>
@@ -4699,7 +4699,7 @@
         <v>22</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>1325</v>
+        <v>1324</v>
       </c>
       <c r="H4" s="5" t="s">
         <v>108</v>
@@ -4731,7 +4731,7 @@
         <v>24</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>1326</v>
+        <v>1325</v>
       </c>
       <c r="H5" s="5" t="s">
         <v>113</v>
@@ -4763,7 +4763,7 @@
         <v>25</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>1327</v>
+        <v>1326</v>
       </c>
       <c r="H6" s="5" t="s">
         <v>118</v>
@@ -4795,7 +4795,7 @@
         <v>27</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>1328</v>
+        <v>1327</v>
       </c>
       <c r="H7" s="5" t="s">
         <v>123</v>
@@ -6534,7 +6534,7 @@
         <v>425</v>
       </c>
       <c r="E65" s="8" t="s">
-        <v>1329</v>
+        <v>1328</v>
       </c>
       <c r="G65" s="5" t="s">
         <v>439</v>
@@ -6604,7 +6604,7 @@
         <v>445</v>
       </c>
       <c r="E67" s="8" t="s">
-        <v>1330</v>
+        <v>1329</v>
       </c>
       <c r="G67" s="5" t="s">
         <v>452</v>
@@ -6738,7 +6738,7 @@
         <v>464</v>
       </c>
       <c r="E71" s="8" t="s">
-        <v>1331</v>
+        <v>1330</v>
       </c>
       <c r="G71" s="5" t="s">
         <v>477</v>
@@ -7632,7 +7632,7 @@
         <v>639</v>
       </c>
       <c r="E98" s="8" t="s">
-        <v>1332</v>
+        <v>1331</v>
       </c>
       <c r="G98" s="5" t="s">
         <v>653</v>
@@ -7734,7 +7734,7 @@
         <v>659</v>
       </c>
       <c r="E101" s="8" t="s">
-        <v>1333</v>
+        <v>1332</v>
       </c>
       <c r="G101" s="5" t="s">
         <v>672</v>
@@ -8729,7 +8729,7 @@
         <v>856</v>
       </c>
       <c r="E132" s="8" t="s">
-        <v>1334</v>
+        <v>1333</v>
       </c>
       <c r="F132" s="5"/>
       <c r="H132" s="5" t="s">
@@ -8849,7 +8849,7 @@
         <v>877</v>
       </c>
       <c r="E136" s="8" t="s">
-        <v>1335</v>
+        <v>1334</v>
       </c>
       <c r="F136" s="5"/>
       <c r="H136" s="5" t="s">
@@ -8969,7 +8969,7 @@
         <v>898</v>
       </c>
       <c r="E140" s="8" t="s">
-        <v>1336</v>
+        <v>1335</v>
       </c>
       <c r="F140" s="5"/>
       <c r="H140" s="5" t="s">
@@ -9089,7 +9089,7 @@
         <v>918</v>
       </c>
       <c r="E144" s="8" t="s">
-        <v>1337</v>
+        <v>1336</v>
       </c>
       <c r="F144" s="5"/>
       <c r="H144" s="5" t="s">
@@ -9200,735 +9200,735 @@
     </row>
     <row r="148" spans="1:13" ht="75" x14ac:dyDescent="0.25">
       <c r="A148" s="7" t="s">
+        <v>939</v>
+      </c>
+      <c r="B148" s="7" t="s">
         <v>940</v>
       </c>
-      <c r="B148" s="7" t="s">
+      <c r="C148" s="7" t="s">
         <v>941</v>
-      </c>
-      <c r="C148" s="7" t="s">
-        <v>942</v>
       </c>
       <c r="D148" s="7"/>
       <c r="E148" s="9" t="s">
-        <v>1338</v>
+        <v>1337</v>
       </c>
       <c r="F148" s="7"/>
       <c r="G148" s="7" t="s">
         <v>485</v>
       </c>
       <c r="H148" s="7" t="s">
+        <v>942</v>
+      </c>
+      <c r="I148" s="7" t="s">
         <v>943</v>
       </c>
-      <c r="I148" s="7" t="s">
+      <c r="J148" s="7" t="s">
         <v>944</v>
       </c>
-      <c r="J148" s="7" t="s">
+      <c r="K148" s="7" t="s">
         <v>945</v>
-      </c>
-      <c r="K148" s="7" t="s">
-        <v>946</v>
       </c>
       <c r="L148" s="7" t="s">
         <v>23</v>
       </c>
       <c r="M148" s="7" t="s">
-        <v>947</v>
+        <v>946</v>
       </c>
     </row>
     <row r="149" spans="1:13" ht="60" x14ac:dyDescent="0.25">
       <c r="A149" s="7" t="s">
-        <v>948</v>
+        <v>947</v>
       </c>
       <c r="B149" s="7" t="s">
+        <v>940</v>
+      </c>
+      <c r="C149" s="7" t="s">
         <v>941</v>
-      </c>
-      <c r="C149" s="7" t="s">
-        <v>942</v>
       </c>
       <c r="D149" s="7"/>
       <c r="E149" s="7"/>
       <c r="F149" s="7"/>
       <c r="G149" s="7" t="s">
+        <v>948</v>
+      </c>
+      <c r="H149" s="7" t="s">
         <v>949</v>
       </c>
-      <c r="H149" s="7" t="s">
+      <c r="I149" s="7" t="s">
         <v>950</v>
       </c>
-      <c r="I149" s="7" t="s">
+      <c r="J149" s="7" t="s">
         <v>951</v>
       </c>
-      <c r="J149" s="7" t="s">
+      <c r="K149" s="7" t="s">
         <v>952</v>
-      </c>
-      <c r="K149" s="7" t="s">
-        <v>953</v>
       </c>
       <c r="L149" s="7" t="s">
         <v>19</v>
       </c>
       <c r="M149" s="7" t="s">
-        <v>954</v>
+        <v>953</v>
       </c>
     </row>
     <row r="150" spans="1:13" ht="75" x14ac:dyDescent="0.25">
       <c r="A150" s="7" t="s">
+        <v>954</v>
+      </c>
+      <c r="B150" s="7" t="s">
+        <v>940</v>
+      </c>
+      <c r="C150" s="7" t="s">
         <v>955</v>
-      </c>
-      <c r="B150" s="7" t="s">
-        <v>941</v>
-      </c>
-      <c r="C150" s="7" t="s">
-        <v>956</v>
       </c>
       <c r="D150" s="7"/>
       <c r="E150" s="9" t="s">
-        <v>1339</v>
+        <v>1338</v>
       </c>
       <c r="F150" s="7"/>
       <c r="G150" s="7" t="s">
+        <v>956</v>
+      </c>
+      <c r="H150" s="7" t="s">
         <v>957</v>
       </c>
-      <c r="H150" s="7" t="s">
+      <c r="I150" s="7" t="s">
         <v>958</v>
       </c>
-      <c r="I150" s="7" t="s">
+      <c r="J150" s="7" t="s">
         <v>959</v>
       </c>
-      <c r="J150" s="7" t="s">
+      <c r="K150" s="7" t="s">
         <v>960</v>
-      </c>
-      <c r="K150" s="7" t="s">
-        <v>961</v>
       </c>
       <c r="L150" s="7" t="s">
         <v>26</v>
       </c>
       <c r="M150" s="7" t="s">
-        <v>962</v>
+        <v>961</v>
       </c>
     </row>
     <row r="151" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A151" s="7" t="s">
-        <v>963</v>
+        <v>962</v>
       </c>
       <c r="B151" s="7" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
       <c r="C151" s="7" t="s">
-        <v>956</v>
+        <v>955</v>
       </c>
       <c r="D151" s="7"/>
       <c r="E151" s="7"/>
       <c r="F151" s="7"/>
       <c r="G151" s="7" t="s">
+        <v>963</v>
+      </c>
+      <c r="H151" s="7" t="s">
         <v>964</v>
       </c>
-      <c r="H151" s="7" t="s">
+      <c r="I151" s="7" t="s">
         <v>965</v>
       </c>
-      <c r="I151" s="7" t="s">
+      <c r="J151" s="7" t="s">
         <v>966</v>
       </c>
-      <c r="J151" s="7" t="s">
+      <c r="K151" s="7" t="s">
         <v>967</v>
-      </c>
-      <c r="K151" s="7" t="s">
-        <v>968</v>
       </c>
       <c r="L151" s="7" t="s">
         <v>23</v>
       </c>
       <c r="M151" s="7" t="s">
-        <v>969</v>
+        <v>968</v>
       </c>
     </row>
     <row r="152" spans="1:13" ht="75" x14ac:dyDescent="0.25">
       <c r="A152" s="7" t="s">
+        <v>969</v>
+      </c>
+      <c r="B152" s="7" t="s">
+        <v>940</v>
+      </c>
+      <c r="C152" s="7" t="s">
         <v>970</v>
-      </c>
-      <c r="B152" s="7" t="s">
-        <v>941</v>
-      </c>
-      <c r="C152" s="7" t="s">
-        <v>971</v>
       </c>
       <c r="D152" s="7"/>
       <c r="E152" s="9" t="s">
-        <v>1340</v>
+        <v>1339</v>
       </c>
       <c r="F152" s="7"/>
       <c r="G152" s="7" t="s">
+        <v>971</v>
+      </c>
+      <c r="H152" s="7" t="s">
         <v>972</v>
       </c>
-      <c r="H152" s="7" t="s">
+      <c r="I152" s="7" t="s">
         <v>973</v>
       </c>
-      <c r="I152" s="7" t="s">
+      <c r="J152" s="7" t="s">
         <v>974</v>
       </c>
-      <c r="J152" s="7" t="s">
+      <c r="K152" s="7" t="s">
         <v>975</v>
-      </c>
-      <c r="K152" s="7" t="s">
-        <v>976</v>
       </c>
       <c r="L152" s="7" t="s">
         <v>23</v>
       </c>
       <c r="M152" s="7" t="s">
-        <v>977</v>
+        <v>976</v>
       </c>
     </row>
     <row r="153" spans="1:13" ht="60" x14ac:dyDescent="0.25">
       <c r="A153" s="7" t="s">
-        <v>978</v>
+        <v>977</v>
       </c>
       <c r="B153" s="7" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
       <c r="C153" s="7" t="s">
-        <v>971</v>
+        <v>970</v>
       </c>
       <c r="D153" s="7"/>
       <c r="E153" s="7"/>
       <c r="F153" s="7"/>
       <c r="G153" s="7" t="s">
+        <v>978</v>
+      </c>
+      <c r="H153" s="7" t="s">
         <v>979</v>
       </c>
-      <c r="H153" s="7" t="s">
+      <c r="I153" s="7" t="s">
         <v>980</v>
       </c>
-      <c r="I153" s="7" t="s">
+      <c r="J153" s="7" t="s">
         <v>981</v>
       </c>
-      <c r="J153" s="7" t="s">
+      <c r="K153" s="7" t="s">
         <v>982</v>
-      </c>
-      <c r="K153" s="7" t="s">
-        <v>983</v>
       </c>
       <c r="L153" s="7" t="s">
         <v>23</v>
       </c>
       <c r="M153" s="7" t="s">
-        <v>984</v>
+        <v>983</v>
       </c>
     </row>
     <row r="154" spans="1:13" ht="75" x14ac:dyDescent="0.25">
       <c r="A154" s="7" t="s">
+        <v>984</v>
+      </c>
+      <c r="B154" s="7" t="s">
+        <v>940</v>
+      </c>
+      <c r="C154" s="7" t="s">
         <v>985</v>
-      </c>
-      <c r="B154" s="7" t="s">
-        <v>941</v>
-      </c>
-      <c r="C154" s="7" t="s">
-        <v>986</v>
       </c>
       <c r="D154" s="7"/>
       <c r="E154" s="9" t="s">
-        <v>1341</v>
+        <v>1340</v>
       </c>
       <c r="F154" s="7"/>
       <c r="G154" s="7" t="s">
+        <v>986</v>
+      </c>
+      <c r="H154" s="7" t="s">
         <v>987</v>
       </c>
-      <c r="H154" s="7" t="s">
+      <c r="I154" s="7" t="s">
         <v>988</v>
       </c>
-      <c r="I154" s="7" t="s">
+      <c r="J154" s="7" t="s">
         <v>989</v>
       </c>
-      <c r="J154" s="7" t="s">
+      <c r="K154" s="7" t="s">
         <v>990</v>
-      </c>
-      <c r="K154" s="7" t="s">
-        <v>991</v>
       </c>
       <c r="L154" s="7" t="s">
         <v>19</v>
       </c>
       <c r="M154" s="7" t="s">
-        <v>992</v>
+        <v>991</v>
       </c>
     </row>
     <row r="155" spans="1:13" ht="60" x14ac:dyDescent="0.25">
       <c r="A155" s="7" t="s">
-        <v>993</v>
+        <v>992</v>
       </c>
       <c r="B155" s="7" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
       <c r="C155" s="7" t="s">
-        <v>986</v>
+        <v>985</v>
       </c>
       <c r="D155" s="7"/>
       <c r="E155" s="7"/>
       <c r="F155" s="7"/>
       <c r="G155" s="7" t="s">
+        <v>993</v>
+      </c>
+      <c r="H155" s="7" t="s">
         <v>994</v>
       </c>
-      <c r="H155" s="7" t="s">
+      <c r="I155" s="7" t="s">
         <v>995</v>
       </c>
-      <c r="I155" s="7" t="s">
+      <c r="J155" s="7" t="s">
         <v>996</v>
       </c>
-      <c r="J155" s="7" t="s">
+      <c r="K155" s="7" t="s">
         <v>997</v>
-      </c>
-      <c r="K155" s="7" t="s">
-        <v>998</v>
       </c>
       <c r="L155" s="7" t="s">
         <v>21</v>
       </c>
       <c r="M155" s="7" t="s">
-        <v>999</v>
+        <v>998</v>
       </c>
     </row>
     <row r="156" spans="1:13" ht="75" x14ac:dyDescent="0.25">
       <c r="A156" s="7" t="s">
+        <v>999</v>
+      </c>
+      <c r="B156" s="7" t="s">
+        <v>940</v>
+      </c>
+      <c r="C156" s="7" t="s">
         <v>1000</v>
-      </c>
-      <c r="B156" s="7" t="s">
-        <v>941</v>
-      </c>
-      <c r="C156" s="7" t="s">
-        <v>1001</v>
       </c>
       <c r="D156" s="7"/>
       <c r="E156" s="9" t="s">
-        <v>1342</v>
+        <v>1341</v>
       </c>
       <c r="F156" s="7"/>
       <c r="G156" s="7" t="s">
+        <v>1001</v>
+      </c>
+      <c r="H156" s="7" t="s">
         <v>1002</v>
       </c>
-      <c r="H156" s="7" t="s">
+      <c r="I156" s="7" t="s">
         <v>1003</v>
       </c>
-      <c r="I156" s="7" t="s">
+      <c r="J156" s="7" t="s">
         <v>1004</v>
       </c>
-      <c r="J156" s="7" t="s">
+      <c r="K156" s="7" t="s">
         <v>1005</v>
-      </c>
-      <c r="K156" s="7" t="s">
-        <v>1006</v>
       </c>
       <c r="L156" s="7" t="s">
         <v>19</v>
       </c>
       <c r="M156" s="7" t="s">
-        <v>1007</v>
+        <v>1006</v>
       </c>
     </row>
     <row r="157" spans="1:13" ht="60" x14ac:dyDescent="0.25">
       <c r="A157" s="7" t="s">
-        <v>1008</v>
+        <v>1007</v>
       </c>
       <c r="B157" s="7" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
       <c r="C157" s="7" t="s">
-        <v>1001</v>
+        <v>1000</v>
       </c>
       <c r="D157" s="7"/>
       <c r="E157" s="7"/>
       <c r="F157" s="7"/>
       <c r="G157" s="7" t="s">
+        <v>1008</v>
+      </c>
+      <c r="H157" s="7" t="s">
         <v>1009</v>
       </c>
-      <c r="H157" s="7" t="s">
+      <c r="I157" s="7" t="s">
         <v>1010</v>
       </c>
-      <c r="I157" s="7" t="s">
+      <c r="J157" s="7" t="s">
         <v>1011</v>
       </c>
-      <c r="J157" s="7" t="s">
+      <c r="K157" s="7" t="s">
         <v>1012</v>
-      </c>
-      <c r="K157" s="7" t="s">
-        <v>1013</v>
       </c>
       <c r="L157" s="7" t="s">
         <v>23</v>
       </c>
       <c r="M157" s="7" t="s">
-        <v>1014</v>
+        <v>1013</v>
       </c>
     </row>
     <row r="158" spans="1:13" ht="45" x14ac:dyDescent="0.25">
       <c r="A158" s="7" t="s">
-        <v>1015</v>
+        <v>1014</v>
       </c>
       <c r="B158" s="7" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
       <c r="C158" s="7" t="s">
-        <v>1001</v>
+        <v>1000</v>
       </c>
       <c r="D158" s="7"/>
       <c r="E158" s="7"/>
       <c r="F158" s="7"/>
       <c r="G158" s="7" t="s">
+        <v>1015</v>
+      </c>
+      <c r="H158" s="7" t="s">
         <v>1016</v>
       </c>
-      <c r="H158" s="7" t="s">
+      <c r="I158" s="7" t="s">
         <v>1017</v>
       </c>
-      <c r="I158" s="7" t="s">
+      <c r="J158" s="7" t="s">
         <v>1018</v>
       </c>
-      <c r="J158" s="7" t="s">
+      <c r="K158" s="7" t="s">
         <v>1019</v>
-      </c>
-      <c r="K158" s="7" t="s">
-        <v>1020</v>
       </c>
       <c r="L158" s="7" t="s">
         <v>26</v>
       </c>
       <c r="M158" s="7" t="s">
-        <v>1021</v>
+        <v>1020</v>
       </c>
     </row>
     <row r="159" spans="1:13" ht="75" x14ac:dyDescent="0.25">
       <c r="A159" s="7" t="s">
+        <v>1021</v>
+      </c>
+      <c r="B159" s="7" t="s">
+        <v>940</v>
+      </c>
+      <c r="C159" s="7" t="s">
         <v>1022</v>
-      </c>
-      <c r="B159" s="7" t="s">
-        <v>941</v>
-      </c>
-      <c r="C159" s="7" t="s">
-        <v>1023</v>
       </c>
       <c r="D159" s="7"/>
       <c r="E159" s="9" t="s">
-        <v>1343</v>
+        <v>1342</v>
       </c>
       <c r="F159" s="7"/>
       <c r="G159" s="7" t="s">
+        <v>1023</v>
+      </c>
+      <c r="H159" s="7" t="s">
         <v>1024</v>
       </c>
-      <c r="H159" s="7" t="s">
+      <c r="I159" s="7" t="s">
         <v>1025</v>
       </c>
-      <c r="I159" s="7" t="s">
+      <c r="J159" s="7" t="s">
         <v>1026</v>
       </c>
-      <c r="J159" s="7" t="s">
+      <c r="K159" s="7" t="s">
         <v>1027</v>
-      </c>
-      <c r="K159" s="7" t="s">
-        <v>1028</v>
       </c>
       <c r="L159" s="7" t="s">
         <v>21</v>
       </c>
       <c r="M159" s="7" t="s">
-        <v>1029</v>
+        <v>1028</v>
       </c>
     </row>
     <row r="160" spans="1:13" ht="75" x14ac:dyDescent="0.25">
       <c r="A160" s="7" t="s">
-        <v>1030</v>
+        <v>1029</v>
       </c>
       <c r="B160" s="7" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
       <c r="C160" s="7" t="s">
-        <v>1023</v>
+        <v>1022</v>
       </c>
       <c r="D160" s="7"/>
       <c r="E160" s="7"/>
       <c r="F160" s="7"/>
       <c r="G160" s="7" t="s">
+        <v>1030</v>
+      </c>
+      <c r="H160" s="7" t="s">
         <v>1031</v>
       </c>
-      <c r="H160" s="7" t="s">
+      <c r="I160" s="7" t="s">
         <v>1032</v>
       </c>
-      <c r="I160" s="7" t="s">
+      <c r="J160" s="7" t="s">
         <v>1033</v>
       </c>
-      <c r="J160" s="7" t="s">
+      <c r="K160" s="7" t="s">
         <v>1034</v>
-      </c>
-      <c r="K160" s="7" t="s">
-        <v>1035</v>
       </c>
       <c r="L160" s="7" t="s">
         <v>21</v>
       </c>
       <c r="M160" s="7" t="s">
-        <v>1036</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="161" spans="1:13" ht="45" x14ac:dyDescent="0.25">
       <c r="A161" s="7" t="s">
-        <v>1037</v>
+        <v>1036</v>
       </c>
       <c r="B161" s="7" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
       <c r="C161" s="7" t="s">
-        <v>1023</v>
+        <v>1022</v>
       </c>
       <c r="D161" s="7"/>
       <c r="E161" s="7"/>
       <c r="F161" s="7"/>
       <c r="G161" s="7" t="s">
+        <v>1037</v>
+      </c>
+      <c r="H161" s="7" t="s">
         <v>1038</v>
       </c>
-      <c r="H161" s="7" t="s">
+      <c r="I161" s="7" t="s">
         <v>1039</v>
       </c>
-      <c r="I161" s="7" t="s">
+      <c r="J161" s="7" t="s">
         <v>1040</v>
       </c>
-      <c r="J161" s="7" t="s">
+      <c r="K161" s="7" t="s">
         <v>1041</v>
-      </c>
-      <c r="K161" s="7" t="s">
-        <v>1042</v>
       </c>
       <c r="L161" s="7" t="s">
         <v>26</v>
       </c>
       <c r="M161" s="7" t="s">
-        <v>1043</v>
+        <v>1042</v>
       </c>
     </row>
     <row r="162" spans="1:13" ht="75" x14ac:dyDescent="0.25">
       <c r="A162" s="7" t="s">
+        <v>1043</v>
+      </c>
+      <c r="B162" s="7" t="s">
+        <v>940</v>
+      </c>
+      <c r="C162" s="7" t="s">
         <v>1044</v>
-      </c>
-      <c r="B162" s="7" t="s">
-        <v>941</v>
-      </c>
-      <c r="C162" s="7" t="s">
-        <v>1045</v>
       </c>
       <c r="D162" s="7"/>
       <c r="E162" s="9" t="s">
-        <v>1344</v>
+        <v>1343</v>
       </c>
       <c r="F162" s="7"/>
       <c r="G162" s="7" t="s">
         <v>91</v>
       </c>
       <c r="H162" s="7" t="s">
+        <v>1045</v>
+      </c>
+      <c r="I162" s="7" t="s">
         <v>1046</v>
       </c>
-      <c r="I162" s="7" t="s">
+      <c r="J162" s="7" t="s">
         <v>1047</v>
       </c>
-      <c r="J162" s="7" t="s">
+      <c r="K162" s="7" t="s">
         <v>1048</v>
-      </c>
-      <c r="K162" s="7" t="s">
-        <v>1049</v>
       </c>
       <c r="L162" s="7" t="s">
         <v>23</v>
       </c>
       <c r="M162" s="7" t="s">
-        <v>1050</v>
+        <v>1049</v>
       </c>
     </row>
     <row r="163" spans="1:13" ht="75" x14ac:dyDescent="0.25">
       <c r="A163" s="7" t="s">
-        <v>1051</v>
+        <v>1050</v>
       </c>
       <c r="B163" s="7" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
       <c r="C163" s="7" t="s">
-        <v>1045</v>
+        <v>1044</v>
       </c>
       <c r="D163" s="7"/>
       <c r="E163" s="7"/>
       <c r="F163" s="7"/>
       <c r="G163" s="7" t="s">
+        <v>1051</v>
+      </c>
+      <c r="H163" s="7" t="s">
         <v>1052</v>
       </c>
-      <c r="H163" s="7" t="s">
+      <c r="I163" s="7" t="s">
         <v>1053</v>
       </c>
-      <c r="I163" s="7" t="s">
+      <c r="J163" s="7" t="s">
         <v>1054</v>
       </c>
-      <c r="J163" s="7" t="s">
+      <c r="K163" s="7" t="s">
         <v>1055</v>
-      </c>
-      <c r="K163" s="7" t="s">
-        <v>1056</v>
       </c>
       <c r="L163" s="7" t="s">
         <v>19</v>
       </c>
       <c r="M163" s="7" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="164" spans="1:13" ht="60" x14ac:dyDescent="0.25">
       <c r="A164" s="7" t="s">
-        <v>1058</v>
+        <v>1057</v>
       </c>
       <c r="B164" s="7" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
       <c r="C164" s="7" t="s">
-        <v>1045</v>
+        <v>1044</v>
       </c>
       <c r="D164" s="7"/>
       <c r="E164" s="7"/>
       <c r="F164" s="7"/>
       <c r="G164" s="7" t="s">
+        <v>1058</v>
+      </c>
+      <c r="H164" s="7" t="s">
         <v>1059</v>
       </c>
-      <c r="H164" s="7" t="s">
+      <c r="I164" s="7" t="s">
         <v>1060</v>
       </c>
-      <c r="I164" s="7" t="s">
+      <c r="J164" s="7" t="s">
         <v>1061</v>
       </c>
-      <c r="J164" s="7" t="s">
+      <c r="K164" s="7" t="s">
         <v>1062</v>
-      </c>
-      <c r="K164" s="7" t="s">
-        <v>1063</v>
       </c>
       <c r="L164" s="7" t="s">
         <v>26</v>
       </c>
       <c r="M164" s="7" t="s">
-        <v>1064</v>
+        <v>1063</v>
       </c>
     </row>
     <row r="165" spans="1:13" ht="60" x14ac:dyDescent="0.25">
       <c r="A165" s="7" t="s">
-        <v>1065</v>
+        <v>1064</v>
       </c>
       <c r="B165" s="7" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
       <c r="C165" s="7" t="s">
-        <v>1045</v>
+        <v>1044</v>
       </c>
       <c r="D165" s="7"/>
       <c r="E165" s="7"/>
       <c r="F165" s="7"/>
       <c r="G165" s="7" t="s">
+        <v>1065</v>
+      </c>
+      <c r="H165" s="7" t="s">
         <v>1066</v>
       </c>
-      <c r="H165" s="7" t="s">
+      <c r="I165" s="7" t="s">
         <v>1067</v>
       </c>
-      <c r="I165" s="7" t="s">
+      <c r="J165" s="7" t="s">
         <v>1068</v>
       </c>
-      <c r="J165" s="7" t="s">
+      <c r="K165" s="7" t="s">
         <v>1069</v>
-      </c>
-      <c r="K165" s="7" t="s">
-        <v>1070</v>
       </c>
       <c r="L165" s="7" t="s">
         <v>19</v>
       </c>
       <c r="M165" s="7" t="s">
-        <v>1071</v>
+        <v>1070</v>
       </c>
     </row>
     <row r="166" spans="1:13" ht="75" x14ac:dyDescent="0.25">
       <c r="A166" s="7" t="s">
+        <v>1071</v>
+      </c>
+      <c r="B166" s="7" t="s">
+        <v>940</v>
+      </c>
+      <c r="C166" s="7" t="s">
         <v>1072</v>
-      </c>
-      <c r="B166" s="7" t="s">
-        <v>941</v>
-      </c>
-      <c r="C166" s="7" t="s">
-        <v>1073</v>
       </c>
       <c r="D166" s="7"/>
       <c r="E166" s="9" t="s">
-        <v>1345</v>
+        <v>1344</v>
       </c>
       <c r="F166" s="7"/>
       <c r="G166" s="7" t="s">
+        <v>1073</v>
+      </c>
+      <c r="H166" s="7" t="s">
         <v>1074</v>
       </c>
-      <c r="H166" s="7" t="s">
+      <c r="I166" s="7" t="s">
         <v>1075</v>
       </c>
-      <c r="I166" s="7" t="s">
+      <c r="J166" s="7" t="s">
         <v>1076</v>
       </c>
-      <c r="J166" s="7" t="s">
+      <c r="K166" s="7" t="s">
         <v>1077</v>
-      </c>
-      <c r="K166" s="7" t="s">
-        <v>1078</v>
       </c>
       <c r="L166" s="7" t="s">
         <v>21</v>
       </c>
       <c r="M166" s="7" t="s">
-        <v>1079</v>
+        <v>1078</v>
       </c>
     </row>
     <row r="167" spans="1:13" ht="45" x14ac:dyDescent="0.25">
       <c r="A167" s="7" t="s">
-        <v>1080</v>
+        <v>1079</v>
       </c>
       <c r="B167" s="7" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
       <c r="C167" s="7" t="s">
-        <v>1073</v>
+        <v>1072</v>
       </c>
       <c r="D167" s="7"/>
       <c r="E167" s="7"/>
       <c r="F167" s="7"/>
       <c r="G167" s="7" t="s">
+        <v>1080</v>
+      </c>
+      <c r="H167" s="7" t="s">
         <v>1081</v>
       </c>
-      <c r="H167" s="7" t="s">
+      <c r="I167" s="7" t="s">
         <v>1082</v>
       </c>
-      <c r="I167" s="7" t="s">
+      <c r="J167" s="7" t="s">
         <v>1083</v>
       </c>
-      <c r="J167" s="7" t="s">
+      <c r="K167" s="7" t="s">
         <v>1084</v>
-      </c>
-      <c r="K167" s="7" t="s">
-        <v>1085</v>
       </c>
       <c r="L167" s="7" t="s">
         <v>19</v>
       </c>
       <c r="M167" s="7" t="s">
-        <v>1086</v>
+        <v>1085</v>
       </c>
     </row>
     <row r="168" spans="1:13" ht="90" x14ac:dyDescent="0.25">
       <c r="A168" s="7" t="s">
-        <v>1087</v>
+        <v>1086</v>
       </c>
       <c r="B168" s="7" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
       <c r="C168" s="7" t="s">
-        <v>1073</v>
+        <v>1072</v>
       </c>
       <c r="D168" s="7"/>
       <c r="E168" s="7"/>
       <c r="F168" s="7"/>
       <c r="G168" s="7" t="s">
-        <v>1088</v>
+        <v>1087</v>
       </c>
       <c r="H168" s="7" t="s">
         <v>92</v>
@@ -9946,131 +9946,131 @@
         <v>19</v>
       </c>
       <c r="M168" s="7" t="s">
-        <v>1089</v>
+        <v>1088</v>
       </c>
     </row>
     <row r="169" spans="1:13" ht="75" x14ac:dyDescent="0.25">
       <c r="A169" s="7" t="s">
+        <v>1089</v>
+      </c>
+      <c r="B169" s="7" t="s">
+        <v>940</v>
+      </c>
+      <c r="C169" s="7" t="s">
         <v>1090</v>
-      </c>
-      <c r="B169" s="7" t="s">
-        <v>941</v>
-      </c>
-      <c r="C169" s="7" t="s">
-        <v>1091</v>
       </c>
       <c r="D169" s="7"/>
       <c r="E169" s="9" t="s">
-        <v>1346</v>
+        <v>1345</v>
       </c>
       <c r="F169" s="7"/>
       <c r="G169" s="7" t="s">
+        <v>1091</v>
+      </c>
+      <c r="H169" s="7" t="s">
         <v>1092</v>
       </c>
-      <c r="H169" s="7" t="s">
+      <c r="I169" s="7" t="s">
         <v>1093</v>
       </c>
-      <c r="I169" s="7" t="s">
+      <c r="J169" s="7" t="s">
         <v>1094</v>
       </c>
-      <c r="J169" s="7" t="s">
+      <c r="K169" s="7" t="s">
         <v>1095</v>
-      </c>
-      <c r="K169" s="7" t="s">
-        <v>1096</v>
       </c>
       <c r="L169" s="7" t="s">
         <v>23</v>
       </c>
       <c r="M169" s="7" t="s">
-        <v>1097</v>
+        <v>1096</v>
       </c>
     </row>
     <row r="170" spans="1:13" ht="60" x14ac:dyDescent="0.25">
       <c r="A170" s="7" t="s">
-        <v>1098</v>
+        <v>1097</v>
       </c>
       <c r="B170" s="7" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
       <c r="C170" s="7" t="s">
-        <v>1091</v>
+        <v>1090</v>
       </c>
       <c r="D170" s="7"/>
       <c r="E170" s="7"/>
       <c r="F170" s="7"/>
       <c r="G170" s="7" t="s">
+        <v>1098</v>
+      </c>
+      <c r="H170" s="7" t="s">
         <v>1099</v>
       </c>
-      <c r="H170" s="7" t="s">
+      <c r="I170" s="7" t="s">
         <v>1100</v>
       </c>
-      <c r="I170" s="7" t="s">
+      <c r="J170" s="7" t="s">
         <v>1101</v>
       </c>
-      <c r="J170" s="7" t="s">
+      <c r="K170" s="7" t="s">
         <v>1102</v>
-      </c>
-      <c r="K170" s="7" t="s">
-        <v>1103</v>
       </c>
       <c r="L170" s="7" t="s">
         <v>21</v>
       </c>
       <c r="M170" s="7" t="s">
-        <v>1104</v>
+        <v>1103</v>
       </c>
     </row>
     <row r="171" spans="1:13" ht="45" x14ac:dyDescent="0.25">
       <c r="A171" s="7" t="s">
-        <v>1105</v>
+        <v>1104</v>
       </c>
       <c r="B171" s="7" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
       <c r="C171" s="7" t="s">
-        <v>1091</v>
+        <v>1090</v>
       </c>
       <c r="D171" s="7"/>
       <c r="E171" s="7"/>
       <c r="F171" s="7"/>
       <c r="G171" s="7" t="s">
+        <v>1105</v>
+      </c>
+      <c r="H171" s="7" t="s">
         <v>1106</v>
       </c>
-      <c r="H171" s="7" t="s">
+      <c r="I171" s="7" t="s">
         <v>1107</v>
       </c>
-      <c r="I171" s="7" t="s">
+      <c r="J171" s="7" t="s">
         <v>1108</v>
       </c>
-      <c r="J171" s="7" t="s">
+      <c r="K171" s="7" t="s">
         <v>1109</v>
-      </c>
-      <c r="K171" s="7" t="s">
-        <v>1110</v>
       </c>
       <c r="L171" s="7" t="s">
         <v>19</v>
       </c>
       <c r="M171" s="7" t="s">
-        <v>1111</v>
+        <v>1110</v>
       </c>
     </row>
     <row r="172" spans="1:13" ht="75" x14ac:dyDescent="0.25">
       <c r="A172" s="7" t="s">
-        <v>1112</v>
+        <v>1111</v>
       </c>
       <c r="B172" s="7" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
       <c r="C172" s="7" t="s">
-        <v>1091</v>
+        <v>1090</v>
       </c>
       <c r="D172" s="7"/>
       <c r="E172" s="7"/>
       <c r="F172" s="7"/>
       <c r="G172" s="7" t="s">
-        <v>1113</v>
+        <v>1112</v>
       </c>
       <c r="H172" s="7" t="s">
         <v>92</v>
@@ -10088,1034 +10088,1034 @@
         <v>21</v>
       </c>
       <c r="M172" s="7" t="s">
-        <v>1114</v>
+        <v>1113</v>
       </c>
     </row>
     <row r="173" spans="1:13" ht="75" x14ac:dyDescent="0.25">
       <c r="A173" s="7" t="s">
+        <v>1114</v>
+      </c>
+      <c r="B173" s="7" t="s">
+        <v>940</v>
+      </c>
+      <c r="C173" s="7" t="s">
         <v>1115</v>
-      </c>
-      <c r="B173" s="7" t="s">
-        <v>941</v>
-      </c>
-      <c r="C173" s="7" t="s">
-        <v>1116</v>
       </c>
       <c r="D173" s="7"/>
       <c r="E173" s="9" t="s">
-        <v>1347</v>
+        <v>1346</v>
       </c>
       <c r="F173" s="7"/>
       <c r="G173" s="7" t="s">
+        <v>1116</v>
+      </c>
+      <c r="H173" s="7" t="s">
         <v>1117</v>
       </c>
-      <c r="H173" s="7" t="s">
+      <c r="I173" s="7" t="s">
         <v>1118</v>
       </c>
-      <c r="I173" s="7" t="s">
+      <c r="J173" s="7" t="s">
         <v>1119</v>
       </c>
-      <c r="J173" s="7" t="s">
+      <c r="K173" s="7" t="s">
         <v>1120</v>
-      </c>
-      <c r="K173" s="7" t="s">
-        <v>1121</v>
       </c>
       <c r="L173" s="7" t="s">
         <v>23</v>
       </c>
       <c r="M173" s="7" t="s">
-        <v>1122</v>
+        <v>1121</v>
       </c>
     </row>
     <row r="174" spans="1:13" ht="60" x14ac:dyDescent="0.25">
       <c r="A174" s="7" t="s">
-        <v>1123</v>
+        <v>1122</v>
       </c>
       <c r="B174" s="7" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
       <c r="C174" s="7" t="s">
-        <v>1116</v>
+        <v>1115</v>
       </c>
       <c r="D174" s="7"/>
       <c r="E174" s="7"/>
       <c r="F174" s="7"/>
       <c r="G174" s="7" t="s">
+        <v>1123</v>
+      </c>
+      <c r="H174" s="7" t="s">
         <v>1124</v>
       </c>
-      <c r="H174" s="7" t="s">
+      <c r="I174" s="7" t="s">
         <v>1125</v>
       </c>
-      <c r="I174" s="7" t="s">
+      <c r="J174" s="7" t="s">
         <v>1126</v>
       </c>
-      <c r="J174" s="7" t="s">
+      <c r="K174" s="7" t="s">
         <v>1127</v>
-      </c>
-      <c r="K174" s="7" t="s">
-        <v>1128</v>
       </c>
       <c r="L174" s="7" t="s">
         <v>26</v>
       </c>
       <c r="M174" s="7" t="s">
-        <v>1129</v>
+        <v>1128</v>
       </c>
     </row>
     <row r="175" spans="1:13" ht="75" x14ac:dyDescent="0.25">
       <c r="A175" s="7" t="s">
-        <v>1130</v>
+        <v>1129</v>
       </c>
       <c r="B175" s="7" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
       <c r="C175" s="7" t="s">
-        <v>1116</v>
+        <v>1115</v>
       </c>
       <c r="D175" s="7"/>
       <c r="E175" s="7"/>
       <c r="F175" s="7"/>
       <c r="G175" s="7" t="s">
+        <v>1130</v>
+      </c>
+      <c r="H175" s="7" t="s">
         <v>1131</v>
       </c>
-      <c r="H175" s="7" t="s">
+      <c r="I175" s="7" t="s">
         <v>1132</v>
       </c>
-      <c r="I175" s="7" t="s">
+      <c r="J175" s="7" t="s">
         <v>1133</v>
       </c>
-      <c r="J175" s="7" t="s">
+      <c r="K175" s="7" t="s">
         <v>1134</v>
-      </c>
-      <c r="K175" s="7" t="s">
-        <v>1135</v>
       </c>
       <c r="L175" s="7" t="s">
         <v>21</v>
       </c>
       <c r="M175" s="7" t="s">
-        <v>1136</v>
+        <v>1135</v>
       </c>
     </row>
     <row r="176" spans="1:13" ht="60" x14ac:dyDescent="0.25">
       <c r="A176" s="7" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
       <c r="B176" s="7" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
       <c r="C176" s="7" t="s">
-        <v>1116</v>
+        <v>1115</v>
       </c>
       <c r="D176" s="7"/>
       <c r="E176" s="7"/>
       <c r="F176" s="7"/>
       <c r="G176" s="7" t="s">
+        <v>1137</v>
+      </c>
+      <c r="H176" s="7" t="s">
         <v>1138</v>
       </c>
-      <c r="H176" s="7" t="s">
+      <c r="I176" s="7" t="s">
         <v>1139</v>
       </c>
-      <c r="I176" s="7" t="s">
+      <c r="J176" s="7" t="s">
         <v>1140</v>
       </c>
-      <c r="J176" s="7" t="s">
+      <c r="K176" s="7" t="s">
         <v>1141</v>
-      </c>
-      <c r="K176" s="7" t="s">
-        <v>1142</v>
       </c>
       <c r="L176" s="7" t="s">
         <v>26</v>
       </c>
       <c r="M176" s="7" t="s">
-        <v>1143</v>
+        <v>1142</v>
       </c>
     </row>
     <row r="177" spans="1:13" ht="150" x14ac:dyDescent="0.25">
       <c r="A177" s="7" t="s">
+        <v>1143</v>
+      </c>
+      <c r="B177" s="7" t="s">
+        <v>940</v>
+      </c>
+      <c r="C177" s="7" t="s">
         <v>1144</v>
-      </c>
-      <c r="B177" s="7" t="s">
-        <v>941</v>
-      </c>
-      <c r="C177" s="7" t="s">
-        <v>1145</v>
       </c>
       <c r="D177" s="7"/>
       <c r="E177" s="7" t="s">
-        <v>1348</v>
+        <v>1347</v>
       </c>
       <c r="F177" s="7"/>
       <c r="G177" s="7" t="s">
+        <v>1145</v>
+      </c>
+      <c r="H177" s="7" t="s">
         <v>1146</v>
       </c>
-      <c r="H177" s="7" t="s">
+      <c r="I177" s="7" t="s">
         <v>1147</v>
       </c>
-      <c r="I177" s="7" t="s">
+      <c r="J177" s="7" t="s">
         <v>1148</v>
       </c>
-      <c r="J177" s="7" t="s">
+      <c r="K177" s="7" t="s">
         <v>1149</v>
-      </c>
-      <c r="K177" s="7" t="s">
-        <v>1150</v>
       </c>
       <c r="L177" s="7" t="s">
         <v>19</v>
       </c>
       <c r="M177" s="7" t="s">
-        <v>1151</v>
+        <v>1150</v>
       </c>
     </row>
     <row r="178" spans="1:13" ht="60" x14ac:dyDescent="0.25">
       <c r="A178" s="7" t="s">
-        <v>1152</v>
+        <v>1151</v>
       </c>
       <c r="B178" s="7" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
       <c r="C178" s="7" t="s">
-        <v>1145</v>
+        <v>1144</v>
       </c>
       <c r="D178" s="7"/>
       <c r="E178" s="7"/>
       <c r="F178" s="7"/>
       <c r="G178" s="7" t="s">
+        <v>1152</v>
+      </c>
+      <c r="H178" s="7" t="s">
         <v>1153</v>
       </c>
-      <c r="H178" s="7" t="s">
+      <c r="I178" s="7" t="s">
         <v>1154</v>
       </c>
-      <c r="I178" s="7" t="s">
+      <c r="J178" s="7" t="s">
         <v>1155</v>
       </c>
-      <c r="J178" s="7" t="s">
+      <c r="K178" s="7" t="s">
         <v>1156</v>
-      </c>
-      <c r="K178" s="7" t="s">
-        <v>1157</v>
       </c>
       <c r="L178" s="7" t="s">
         <v>21</v>
       </c>
       <c r="M178" s="7" t="s">
-        <v>1158</v>
+        <v>1157</v>
       </c>
     </row>
     <row r="179" spans="1:13" ht="60" x14ac:dyDescent="0.25">
       <c r="A179" s="7" t="s">
-        <v>1159</v>
+        <v>1158</v>
       </c>
       <c r="B179" s="7" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
       <c r="C179" s="7" t="s">
-        <v>1145</v>
+        <v>1144</v>
       </c>
       <c r="D179" s="7"/>
       <c r="E179" s="7"/>
       <c r="F179" s="7"/>
       <c r="G179" s="7" t="s">
+        <v>1159</v>
+      </c>
+      <c r="H179" s="7" t="s">
         <v>1160</v>
       </c>
-      <c r="H179" s="7" t="s">
+      <c r="I179" s="7" t="s">
         <v>1161</v>
       </c>
-      <c r="I179" s="7" t="s">
+      <c r="J179" s="7" t="s">
         <v>1162</v>
       </c>
-      <c r="J179" s="7" t="s">
+      <c r="K179" s="7" t="s">
         <v>1163</v>
-      </c>
-      <c r="K179" s="7" t="s">
-        <v>1164</v>
       </c>
       <c r="L179" s="7" t="s">
         <v>23</v>
       </c>
       <c r="M179" s="7" t="s">
-        <v>1165</v>
+        <v>1164</v>
       </c>
     </row>
     <row r="180" spans="1:13" ht="75" x14ac:dyDescent="0.25">
       <c r="A180" s="7" t="s">
-        <v>1166</v>
+        <v>1165</v>
       </c>
       <c r="B180" s="7" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
       <c r="C180" s="7" t="s">
-        <v>1145</v>
+        <v>1144</v>
       </c>
       <c r="D180" s="7"/>
       <c r="E180" s="7"/>
       <c r="F180" s="7"/>
       <c r="G180" s="7" t="s">
+        <v>1166</v>
+      </c>
+      <c r="H180" s="7" t="s">
         <v>1167</v>
       </c>
-      <c r="H180" s="7" t="s">
+      <c r="I180" s="7" t="s">
         <v>1168</v>
       </c>
-      <c r="I180" s="7" t="s">
+      <c r="J180" s="7" t="s">
         <v>1169</v>
       </c>
-      <c r="J180" s="7" t="s">
+      <c r="K180" s="7" t="s">
         <v>1170</v>
-      </c>
-      <c r="K180" s="7" t="s">
-        <v>1171</v>
       </c>
       <c r="L180" s="7" t="s">
         <v>26</v>
       </c>
       <c r="M180" s="7" t="s">
-        <v>1172</v>
+        <v>1171</v>
       </c>
     </row>
     <row r="181" spans="1:13" ht="90" x14ac:dyDescent="0.25">
       <c r="A181" s="7" t="s">
-        <v>1173</v>
+        <v>1172</v>
       </c>
       <c r="B181" s="7" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
       <c r="C181" s="7" t="s">
-        <v>1145</v>
+        <v>1144</v>
       </c>
       <c r="D181" s="7"/>
       <c r="E181" s="7"/>
       <c r="F181" s="7"/>
       <c r="G181" s="7" t="s">
+        <v>1173</v>
+      </c>
+      <c r="H181" s="7" t="s">
         <v>1174</v>
       </c>
-      <c r="H181" s="7" t="s">
+      <c r="I181" s="7" t="s">
         <v>1175</v>
       </c>
-      <c r="I181" s="7" t="s">
+      <c r="J181" s="7" t="s">
         <v>1176</v>
       </c>
-      <c r="J181" s="7" t="s">
+      <c r="K181" s="7" t="s">
         <v>1177</v>
-      </c>
-      <c r="K181" s="7" t="s">
-        <v>1178</v>
       </c>
       <c r="L181" s="7" t="s">
         <v>23</v>
       </c>
       <c r="M181" s="7" t="s">
-        <v>1179</v>
+        <v>1178</v>
       </c>
     </row>
     <row r="182" spans="1:13" ht="150" x14ac:dyDescent="0.25">
       <c r="A182" s="7" t="s">
+        <v>1179</v>
+      </c>
+      <c r="B182" s="7" t="s">
+        <v>940</v>
+      </c>
+      <c r="C182" s="7" t="s">
         <v>1180</v>
-      </c>
-      <c r="B182" s="7" t="s">
-        <v>941</v>
-      </c>
-      <c r="C182" s="7" t="s">
-        <v>1181</v>
       </c>
       <c r="D182" s="7"/>
       <c r="E182" s="7" t="s">
-        <v>1349</v>
+        <v>1348</v>
       </c>
       <c r="F182" s="7"/>
       <c r="G182" s="7" t="s">
+        <v>1181</v>
+      </c>
+      <c r="H182" s="7" t="s">
         <v>1182</v>
       </c>
-      <c r="H182" s="7" t="s">
+      <c r="I182" s="7" t="s">
         <v>1183</v>
       </c>
-      <c r="I182" s="7" t="s">
+      <c r="J182" s="7" t="s">
         <v>1184</v>
       </c>
-      <c r="J182" s="7" t="s">
+      <c r="K182" s="7" t="s">
         <v>1185</v>
-      </c>
-      <c r="K182" s="7" t="s">
-        <v>1186</v>
       </c>
       <c r="L182" s="7" t="s">
         <v>23</v>
       </c>
       <c r="M182" s="7" t="s">
-        <v>1187</v>
+        <v>1186</v>
       </c>
     </row>
     <row r="183" spans="1:13" ht="90" x14ac:dyDescent="0.25">
       <c r="A183" s="7" t="s">
-        <v>1188</v>
+        <v>1187</v>
       </c>
       <c r="B183" s="7" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
       <c r="C183" s="7" t="s">
-        <v>1181</v>
+        <v>1180</v>
       </c>
       <c r="D183" s="7"/>
       <c r="E183" s="7"/>
       <c r="F183" s="7"/>
       <c r="G183" s="7" t="s">
+        <v>1188</v>
+      </c>
+      <c r="H183" s="7" t="s">
         <v>1189</v>
       </c>
-      <c r="H183" s="7" t="s">
+      <c r="I183" s="7" t="s">
         <v>1190</v>
       </c>
-      <c r="I183" s="7" t="s">
+      <c r="J183" s="7" t="s">
         <v>1191</v>
       </c>
-      <c r="J183" s="7" t="s">
+      <c r="K183" s="7" t="s">
         <v>1192</v>
-      </c>
-      <c r="K183" s="7" t="s">
-        <v>1193</v>
       </c>
       <c r="L183" s="7" t="s">
         <v>21</v>
       </c>
       <c r="M183" s="7" t="s">
-        <v>1194</v>
+        <v>1193</v>
       </c>
     </row>
     <row r="184" spans="1:13" ht="75" x14ac:dyDescent="0.25">
       <c r="A184" s="7" t="s">
-        <v>1195</v>
+        <v>1194</v>
       </c>
       <c r="B184" s="7" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
       <c r="C184" s="7" t="s">
-        <v>1181</v>
+        <v>1180</v>
       </c>
       <c r="D184" s="7"/>
       <c r="E184" s="7"/>
       <c r="F184" s="7"/>
       <c r="G184" s="7" t="s">
+        <v>1195</v>
+      </c>
+      <c r="H184" s="7" t="s">
         <v>1196</v>
       </c>
-      <c r="H184" s="7" t="s">
+      <c r="I184" s="7" t="s">
         <v>1197</v>
       </c>
-      <c r="I184" s="7" t="s">
+      <c r="J184" s="7" t="s">
         <v>1198</v>
       </c>
-      <c r="J184" s="7" t="s">
+      <c r="K184" s="7" t="s">
         <v>1199</v>
-      </c>
-      <c r="K184" s="7" t="s">
-        <v>1200</v>
       </c>
       <c r="L184" s="7" t="s">
         <v>19</v>
       </c>
       <c r="M184" s="7" t="s">
-        <v>1201</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="185" spans="1:13" ht="45" x14ac:dyDescent="0.25">
       <c r="A185" s="7" t="s">
-        <v>1202</v>
+        <v>1201</v>
       </c>
       <c r="B185" s="7" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
       <c r="C185" s="7" t="s">
-        <v>1181</v>
+        <v>1180</v>
       </c>
       <c r="D185" s="7"/>
       <c r="E185" s="7"/>
       <c r="F185" s="7"/>
       <c r="G185" s="7" t="s">
+        <v>1202</v>
+      </c>
+      <c r="H185" s="7" t="s">
         <v>1203</v>
       </c>
-      <c r="H185" s="7" t="s">
+      <c r="I185" s="7" t="s">
         <v>1204</v>
       </c>
-      <c r="I185" s="7" t="s">
+      <c r="J185" s="7" t="s">
         <v>1205</v>
       </c>
-      <c r="J185" s="7" t="s">
+      <c r="K185" s="7" t="s">
         <v>1206</v>
-      </c>
-      <c r="K185" s="7" t="s">
-        <v>1207</v>
       </c>
       <c r="L185" s="7" t="s">
         <v>19</v>
       </c>
       <c r="M185" s="7" t="s">
-        <v>1208</v>
+        <v>1207</v>
       </c>
     </row>
     <row r="186" spans="1:13" ht="75" x14ac:dyDescent="0.25">
       <c r="A186" s="7" t="s">
-        <v>1209</v>
+        <v>1208</v>
       </c>
       <c r="B186" s="7" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
       <c r="C186" s="7" t="s">
-        <v>1181</v>
+        <v>1180</v>
       </c>
       <c r="D186" s="7"/>
       <c r="E186" s="7"/>
       <c r="F186" s="7"/>
       <c r="G186" s="7" t="s">
+        <v>1209</v>
+      </c>
+      <c r="H186" s="7" t="s">
         <v>1210</v>
       </c>
-      <c r="H186" s="7" t="s">
+      <c r="I186" s="7" t="s">
         <v>1211</v>
       </c>
-      <c r="I186" s="7" t="s">
+      <c r="J186" s="7" t="s">
         <v>1212</v>
       </c>
-      <c r="J186" s="7" t="s">
+      <c r="K186" s="7" t="s">
         <v>1213</v>
-      </c>
-      <c r="K186" s="7" t="s">
-        <v>1214</v>
       </c>
       <c r="L186" s="7" t="s">
         <v>26</v>
       </c>
       <c r="M186" s="7" t="s">
-        <v>1215</v>
+        <v>1214</v>
       </c>
     </row>
     <row r="187" spans="1:13" ht="225" x14ac:dyDescent="0.25">
       <c r="A187" s="7" t="s">
+        <v>1215</v>
+      </c>
+      <c r="B187" s="7" t="s">
+        <v>940</v>
+      </c>
+      <c r="C187" s="7" t="s">
         <v>1216</v>
-      </c>
-      <c r="B187" s="7" t="s">
-        <v>941</v>
-      </c>
-      <c r="C187" s="7" t="s">
-        <v>1217</v>
       </c>
       <c r="D187" s="7"/>
       <c r="E187" s="7" t="s">
-        <v>1352</v>
+        <v>1351</v>
       </c>
       <c r="F187" s="7"/>
       <c r="G187" s="7" t="s">
+        <v>1217</v>
+      </c>
+      <c r="H187" s="7" t="s">
         <v>1218</v>
       </c>
-      <c r="H187" s="7" t="s">
+      <c r="I187" s="7" t="s">
         <v>1219</v>
       </c>
-      <c r="I187" s="7" t="s">
+      <c r="J187" s="7" t="s">
         <v>1220</v>
       </c>
-      <c r="J187" s="7" t="s">
+      <c r="K187" s="7" t="s">
         <v>1221</v>
-      </c>
-      <c r="K187" s="7" t="s">
-        <v>1222</v>
       </c>
       <c r="L187" s="7" t="s">
         <v>26</v>
       </c>
       <c r="M187" s="7" t="s">
-        <v>1223</v>
+        <v>1222</v>
       </c>
     </row>
     <row r="188" spans="1:13" ht="90" x14ac:dyDescent="0.25">
       <c r="A188" s="7" t="s">
-        <v>1224</v>
+        <v>1223</v>
       </c>
       <c r="B188" s="7" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
       <c r="C188" s="7" t="s">
-        <v>1217</v>
+        <v>1216</v>
       </c>
       <c r="D188" s="7"/>
       <c r="E188" s="7"/>
       <c r="F188" s="7"/>
       <c r="G188" s="7" t="s">
+        <v>1224</v>
+      </c>
+      <c r="H188" s="7" t="s">
         <v>1225</v>
       </c>
-      <c r="H188" s="7" t="s">
+      <c r="I188" s="7" t="s">
         <v>1226</v>
       </c>
-      <c r="I188" s="7" t="s">
+      <c r="J188" s="7" t="s">
         <v>1227</v>
       </c>
-      <c r="J188" s="7" t="s">
+      <c r="K188" s="7" t="s">
         <v>1228</v>
-      </c>
-      <c r="K188" s="7" t="s">
-        <v>1229</v>
       </c>
       <c r="L188" s="7" t="s">
         <v>19</v>
       </c>
       <c r="M188" s="7" t="s">
-        <v>1230</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="189" spans="1:13" ht="120" x14ac:dyDescent="0.25">
       <c r="A189" s="7" t="s">
-        <v>1231</v>
+        <v>1230</v>
       </c>
       <c r="B189" s="7" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
       <c r="C189" s="7" t="s">
-        <v>1217</v>
+        <v>1216</v>
       </c>
       <c r="D189" s="7"/>
       <c r="E189" s="7"/>
       <c r="F189" s="7"/>
       <c r="G189" s="7" t="s">
+        <v>1231</v>
+      </c>
+      <c r="H189" s="7" t="s">
         <v>1232</v>
       </c>
-      <c r="H189" s="7" t="s">
+      <c r="I189" s="7" t="s">
         <v>1233</v>
       </c>
-      <c r="I189" s="7" t="s">
+      <c r="J189" s="7" t="s">
         <v>1234</v>
       </c>
-      <c r="J189" s="7" t="s">
+      <c r="K189" s="7" t="s">
         <v>1235</v>
-      </c>
-      <c r="K189" s="7" t="s">
-        <v>1236</v>
       </c>
       <c r="L189" s="7" t="s">
         <v>21</v>
       </c>
       <c r="M189" s="7" t="s">
-        <v>1237</v>
+        <v>1236</v>
       </c>
     </row>
     <row r="190" spans="1:13" ht="60" x14ac:dyDescent="0.25">
       <c r="A190" s="7" t="s">
-        <v>1238</v>
+        <v>1237</v>
       </c>
       <c r="B190" s="7" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
       <c r="C190" s="7" t="s">
-        <v>1217</v>
+        <v>1216</v>
       </c>
       <c r="D190" s="7"/>
       <c r="E190" s="7"/>
       <c r="F190" s="7"/>
       <c r="G190" s="7" t="s">
+        <v>1238</v>
+      </c>
+      <c r="H190" s="7" t="s">
         <v>1239</v>
       </c>
-      <c r="H190" s="7" t="s">
+      <c r="I190" s="7" t="s">
         <v>1240</v>
       </c>
-      <c r="I190" s="7" t="s">
+      <c r="J190" s="7" t="s">
         <v>1241</v>
       </c>
-      <c r="J190" s="7" t="s">
+      <c r="K190" s="7" t="s">
         <v>1242</v>
-      </c>
-      <c r="K190" s="7" t="s">
-        <v>1243</v>
       </c>
       <c r="L190" s="7" t="s">
         <v>19</v>
       </c>
       <c r="M190" s="7" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
     </row>
     <row r="191" spans="1:13" ht="105" x14ac:dyDescent="0.25">
       <c r="A191" s="7" t="s">
-        <v>1245</v>
+        <v>1244</v>
       </c>
       <c r="B191" s="7" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
       <c r="C191" s="7" t="s">
-        <v>1217</v>
+        <v>1216</v>
       </c>
       <c r="D191" s="7"/>
       <c r="E191" s="7"/>
       <c r="F191" s="7"/>
       <c r="G191" s="7" t="s">
+        <v>1245</v>
+      </c>
+      <c r="H191" s="7" t="s">
         <v>1246</v>
       </c>
-      <c r="H191" s="7" t="s">
+      <c r="I191" s="7" t="s">
         <v>1247</v>
       </c>
-      <c r="I191" s="7" t="s">
+      <c r="J191" s="7" t="s">
         <v>1248</v>
       </c>
-      <c r="J191" s="7" t="s">
+      <c r="K191" s="7" t="s">
         <v>1249</v>
-      </c>
-      <c r="K191" s="7" t="s">
-        <v>1250</v>
       </c>
       <c r="L191" s="7" t="s">
         <v>23</v>
       </c>
       <c r="M191" s="7" t="s">
-        <v>1251</v>
+        <v>1250</v>
       </c>
     </row>
     <row r="192" spans="1:13" ht="225" x14ac:dyDescent="0.25">
       <c r="A192" s="7" t="s">
+        <v>1251</v>
+      </c>
+      <c r="B192" s="7" t="s">
+        <v>940</v>
+      </c>
+      <c r="C192" s="7" t="s">
         <v>1252</v>
-      </c>
-      <c r="B192" s="7" t="s">
-        <v>941</v>
-      </c>
-      <c r="C192" s="7" t="s">
-        <v>1253</v>
       </c>
       <c r="D192" s="7"/>
       <c r="E192" s="7" t="s">
-        <v>1350</v>
+        <v>1349</v>
       </c>
       <c r="F192" s="7"/>
       <c r="G192" s="7" t="s">
+        <v>1253</v>
+      </c>
+      <c r="H192" s="7" t="s">
         <v>1254</v>
       </c>
-      <c r="H192" s="7" t="s">
+      <c r="I192" s="7" t="s">
         <v>1255</v>
       </c>
-      <c r="I192" s="7" t="s">
+      <c r="J192" s="7" t="s">
         <v>1256</v>
       </c>
-      <c r="J192" s="7" t="s">
+      <c r="K192" s="7" t="s">
         <v>1257</v>
-      </c>
-      <c r="K192" s="7" t="s">
-        <v>1258</v>
       </c>
       <c r="L192" s="7" t="s">
         <v>19</v>
       </c>
       <c r="M192" s="7" t="s">
-        <v>1259</v>
+        <v>1258</v>
       </c>
     </row>
     <row r="193" spans="1:13" ht="45" x14ac:dyDescent="0.25">
       <c r="A193" s="7" t="s">
-        <v>1260</v>
+        <v>1259</v>
       </c>
       <c r="B193" s="7" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
       <c r="C193" s="7" t="s">
-        <v>1253</v>
+        <v>1252</v>
       </c>
       <c r="D193" s="7"/>
       <c r="E193" s="7"/>
       <c r="F193" s="7"/>
       <c r="G193" s="7" t="s">
+        <v>1260</v>
+      </c>
+      <c r="H193" s="7" t="s">
         <v>1261</v>
       </c>
-      <c r="H193" s="7" t="s">
+      <c r="I193" s="7" t="s">
         <v>1262</v>
       </c>
-      <c r="I193" s="7" t="s">
+      <c r="J193" s="7" t="s">
         <v>1263</v>
       </c>
-      <c r="J193" s="7" t="s">
+      <c r="K193" s="7" t="s">
         <v>1264</v>
-      </c>
-      <c r="K193" s="7" t="s">
-        <v>1265</v>
       </c>
       <c r="L193" s="7" t="s">
         <v>23</v>
       </c>
       <c r="M193" s="7" t="s">
-        <v>1266</v>
+        <v>1265</v>
       </c>
     </row>
     <row r="194" spans="1:13" ht="45" x14ac:dyDescent="0.25">
       <c r="A194" s="7" t="s">
-        <v>1267</v>
+        <v>1266</v>
       </c>
       <c r="B194" s="7" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
       <c r="C194" s="7" t="s">
-        <v>1253</v>
+        <v>1252</v>
       </c>
       <c r="D194" s="7"/>
       <c r="E194" s="7"/>
       <c r="F194" s="7"/>
       <c r="G194" s="7" t="s">
+        <v>1267</v>
+      </c>
+      <c r="H194" s="7" t="s">
         <v>1268</v>
       </c>
-      <c r="H194" s="7" t="s">
+      <c r="I194" s="7" t="s">
         <v>1269</v>
       </c>
-      <c r="I194" s="7" t="s">
+      <c r="J194" s="7" t="s">
         <v>1270</v>
       </c>
-      <c r="J194" s="7" t="s">
+      <c r="K194" s="7" t="s">
         <v>1271</v>
-      </c>
-      <c r="K194" s="7" t="s">
-        <v>1272</v>
       </c>
       <c r="L194" s="7" t="s">
         <v>23</v>
       </c>
       <c r="M194" s="7" t="s">
-        <v>1273</v>
+        <v>1272</v>
       </c>
     </row>
     <row r="195" spans="1:13" ht="45" x14ac:dyDescent="0.25">
       <c r="A195" s="7" t="s">
-        <v>1274</v>
+        <v>1273</v>
       </c>
       <c r="B195" s="7" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
       <c r="C195" s="7" t="s">
-        <v>1253</v>
+        <v>1252</v>
       </c>
       <c r="D195" s="7"/>
       <c r="E195" s="7"/>
       <c r="F195" s="7"/>
       <c r="G195" s="7" t="s">
+        <v>1274</v>
+      </c>
+      <c r="H195" s="7" t="s">
         <v>1275</v>
       </c>
-      <c r="H195" s="7" t="s">
+      <c r="I195" s="7" t="s">
         <v>1276</v>
       </c>
-      <c r="I195" s="7" t="s">
+      <c r="J195" s="7" t="s">
         <v>1277</v>
       </c>
-      <c r="J195" s="7" t="s">
+      <c r="K195" s="7" t="s">
         <v>1278</v>
-      </c>
-      <c r="K195" s="7" t="s">
-        <v>1279</v>
       </c>
       <c r="L195" s="7" t="s">
         <v>26</v>
       </c>
       <c r="M195" s="7" t="s">
-        <v>1280</v>
+        <v>1279</v>
       </c>
     </row>
     <row r="196" spans="1:13" ht="60" x14ac:dyDescent="0.25">
       <c r="A196" s="7" t="s">
-        <v>1281</v>
+        <v>1280</v>
       </c>
       <c r="B196" s="7" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
       <c r="C196" s="7" t="s">
-        <v>1253</v>
+        <v>1252</v>
       </c>
       <c r="D196" s="7"/>
       <c r="E196" s="7"/>
       <c r="F196" s="7"/>
       <c r="G196" s="7" t="s">
+        <v>1281</v>
+      </c>
+      <c r="H196" s="7" t="s">
         <v>1282</v>
       </c>
-      <c r="H196" s="7" t="s">
+      <c r="I196" s="7" t="s">
         <v>1283</v>
       </c>
-      <c r="I196" s="7" t="s">
+      <c r="J196" s="7" t="s">
         <v>1284</v>
       </c>
-      <c r="J196" s="7" t="s">
+      <c r="K196" s="7" t="s">
         <v>1285</v>
-      </c>
-      <c r="K196" s="7" t="s">
-        <v>1286</v>
       </c>
       <c r="L196" s="7" t="s">
         <v>21</v>
       </c>
       <c r="M196" s="7" t="s">
-        <v>1287</v>
+        <v>1286</v>
       </c>
     </row>
     <row r="197" spans="1:13" ht="225" x14ac:dyDescent="0.25">
       <c r="A197" s="7" t="s">
+        <v>1287</v>
+      </c>
+      <c r="B197" s="7" t="s">
+        <v>940</v>
+      </c>
+      <c r="C197" s="7" t="s">
         <v>1288</v>
-      </c>
-      <c r="B197" s="7" t="s">
-        <v>941</v>
-      </c>
-      <c r="C197" s="7" t="s">
-        <v>1289</v>
       </c>
       <c r="D197" s="7"/>
       <c r="E197" s="7" t="s">
-        <v>1351</v>
+        <v>1350</v>
       </c>
       <c r="F197" s="7"/>
       <c r="G197" s="7" t="s">
+        <v>1289</v>
+      </c>
+      <c r="H197" s="7" t="s">
         <v>1290</v>
       </c>
-      <c r="H197" s="7" t="s">
+      <c r="I197" s="7" t="s">
         <v>1291</v>
       </c>
-      <c r="I197" s="7" t="s">
+      <c r="J197" s="7" t="s">
         <v>1292</v>
       </c>
-      <c r="J197" s="7" t="s">
+      <c r="K197" s="7" t="s">
         <v>1293</v>
-      </c>
-      <c r="K197" s="7" t="s">
-        <v>1294</v>
       </c>
       <c r="L197" s="7" t="s">
         <v>23</v>
       </c>
       <c r="M197" s="7" t="s">
-        <v>1295</v>
+        <v>1294</v>
       </c>
     </row>
     <row r="198" spans="1:13" ht="75" x14ac:dyDescent="0.25">
       <c r="A198" s="7" t="s">
-        <v>1296</v>
+        <v>1295</v>
       </c>
       <c r="B198" s="7" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
       <c r="C198" s="7" t="s">
-        <v>1289</v>
+        <v>1288</v>
       </c>
       <c r="D198" s="7"/>
       <c r="E198" s="7"/>
       <c r="F198" s="7"/>
       <c r="G198" s="7" t="s">
+        <v>1296</v>
+      </c>
+      <c r="H198" s="7" t="s">
         <v>1297</v>
       </c>
-      <c r="H198" s="7" t="s">
+      <c r="I198" s="7" t="s">
         <v>1298</v>
       </c>
-      <c r="I198" s="7" t="s">
+      <c r="J198" s="7" t="s">
         <v>1299</v>
       </c>
-      <c r="J198" s="7" t="s">
+      <c r="K198" s="7" t="s">
         <v>1300</v>
-      </c>
-      <c r="K198" s="7" t="s">
-        <v>1301</v>
       </c>
       <c r="L198" s="7" t="s">
         <v>26</v>
       </c>
       <c r="M198" s="7" t="s">
-        <v>1302</v>
+        <v>1301</v>
       </c>
     </row>
     <row r="199" spans="1:13" ht="75" x14ac:dyDescent="0.25">
       <c r="A199" s="7" t="s">
-        <v>1303</v>
+        <v>1302</v>
       </c>
       <c r="B199" s="7" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
       <c r="C199" s="7" t="s">
-        <v>1289</v>
+        <v>1288</v>
       </c>
       <c r="D199" s="7"/>
       <c r="E199" s="7"/>
       <c r="F199" s="7"/>
       <c r="G199" s="7" t="s">
+        <v>1303</v>
+      </c>
+      <c r="H199" s="7" t="s">
         <v>1304</v>
       </c>
-      <c r="H199" s="7" t="s">
+      <c r="I199" s="7" t="s">
         <v>1305</v>
       </c>
-      <c r="I199" s="7" t="s">
+      <c r="J199" s="7" t="s">
         <v>1306</v>
       </c>
-      <c r="J199" s="7" t="s">
+      <c r="K199" s="7" t="s">
         <v>1307</v>
-      </c>
-      <c r="K199" s="7" t="s">
-        <v>1308</v>
       </c>
       <c r="L199" s="7" t="s">
         <v>19</v>
       </c>
       <c r="M199" s="7" t="s">
-        <v>1309</v>
+        <v>1308</v>
       </c>
     </row>
     <row r="200" spans="1:13" ht="105" x14ac:dyDescent="0.25">
       <c r="A200" s="7" t="s">
-        <v>1310</v>
+        <v>1309</v>
       </c>
       <c r="B200" s="7" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
       <c r="C200" s="7" t="s">
-        <v>1289</v>
+        <v>1288</v>
       </c>
       <c r="D200" s="7"/>
       <c r="E200" s="7"/>
       <c r="F200" s="7"/>
       <c r="G200" s="7" t="s">
+        <v>1310</v>
+      </c>
+      <c r="H200" s="7" t="s">
         <v>1311</v>
       </c>
-      <c r="H200" s="7" t="s">
+      <c r="I200" s="7" t="s">
         <v>1312</v>
       </c>
-      <c r="I200" s="7" t="s">
+      <c r="J200" s="7" t="s">
         <v>1313</v>
       </c>
-      <c r="J200" s="7" t="s">
+      <c r="K200" s="7" t="s">
         <v>1314</v>
-      </c>
-      <c r="K200" s="7" t="s">
-        <v>1315</v>
       </c>
       <c r="L200" s="7" t="s">
         <v>21</v>
       </c>
       <c r="M200" s="7" t="s">
-        <v>1316</v>
+        <v>1315</v>
       </c>
     </row>
     <row r="201" spans="1:13" ht="90" x14ac:dyDescent="0.25">
       <c r="A201" s="7" t="s">
-        <v>1317</v>
+        <v>1316</v>
       </c>
       <c r="B201" s="7" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
       <c r="C201" s="7" t="s">
-        <v>1289</v>
+        <v>1288</v>
       </c>
       <c r="D201" s="7"/>
       <c r="E201" s="7"/>
       <c r="F201" s="7"/>
       <c r="G201" s="7" t="s">
+        <v>1317</v>
+      </c>
+      <c r="H201" s="7" t="s">
         <v>1318</v>
       </c>
-      <c r="H201" s="7" t="s">
+      <c r="I201" s="7" t="s">
         <v>1319</v>
       </c>
-      <c r="I201" s="7" t="s">
+      <c r="J201" s="7" t="s">
         <v>1320</v>
       </c>
-      <c r="J201" s="7" t="s">
-        <v>1321</v>
-      </c>
       <c r="K201" s="7" t="s">
-        <v>1301</v>
+        <v>1300</v>
       </c>
       <c r="L201" s="7" t="s">
         <v>23</v>
       </c>
       <c r="M201" s="7" t="s">
-        <v>1322</v>
+        <v>1321</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Thiet ke trang luyen de v19
</commit_message>
<xml_diff>
--- a/ETS2023_Test2_Final_Architecture.xlsx
+++ b/ETS2023_Test2_Final_Architecture.xlsx
@@ -4078,7 +4078,7 @@
     <t>https://raw.githubusercontent.com/bangvang1105-tech/Image-Test-2-ETS-2023/refs/heads/main/p7_186(1).png | https://raw.githubusercontent.com/bangvang1105-tech/Image-Test-2-ETS-2023/refs/heads/main/p7_186(2).png | https://raw.githubusercontent.com/bangvang1105-tech/Image-Test-2-ETS-2023/refs/heads/main/p7_186(3).png</t>
   </si>
   <si>
-    <t>https://drive.google.com/uc?export=view&amp;id=14yGl8HQLGWVQRJ9wKb3tllrgH0prTzdC</t>
+    <t>https://drive.google.com/uc?export=download&amp;id=14yGl8HQLGWVQRJ9wKb3tllrgH0prTzdC</t>
   </si>
 </sst>
 </file>
@@ -4191,7 +4191,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -4214,6 +4214,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -4517,7 +4518,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -4560,11 +4561,12 @@
         <v>200</v>
       </c>
     </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C3" s="10"/>
+    </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="C2" r:id="rId1"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Thiet ke trang luyen de v20
</commit_message>
<xml_diff>
--- a/ETS2023_Test2_Final_Architecture.xlsx
+++ b/ETS2023_Test2_Final_Architecture.xlsx
@@ -4565,8 +4565,11 @@
       <c r="C3" s="10"/>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="C2" r:id="rId1"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId2"/>
 </worksheet>
 </file>
 

</xml_diff>